<commit_message>
Detecteur construit et mesure : R3 a 94 % de precision, 81 % de rappel
Trois regles mesurees sur les verdicts de Vincent (248 paires mesurables,
canal interprofession). Deux decisions issues de l analyse des desaccords :
les videos publiees par un canal vitrine sortent du flux createur (123
paires jugees, dont 116 fausses — un tiers du bruit de l ancien jeu), et
quatre signaux pollueurs mesures sont declasses en faible. R3 depasse les
seuils du contrat mais est calibree sur le meme jeu : a confirmer sur un
lot neuf (critere 6). Mesure : recherche/mesure_detection_2026-09-06.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -473,13 +473,11 @@
           <t>Bigard</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -502,13 +500,11 @@
           <t>Cooperl</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -531,13 +527,11 @@
           <t>Danone</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -560,13 +554,11 @@
           <t>Eurial / Agrial</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -589,13 +581,11 @@
           <t>Groupe Aoste</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -618,13 +608,11 @@
           <t>Groupe Bel</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -647,13 +635,11 @@
           <t>Kermene</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -676,13 +662,11 @@
           <t>LDC</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -705,13 +689,11 @@
           <t>Lactalis</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -734,13 +716,11 @@
           <t>Laita</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -763,13 +743,11 @@
           <t>Pilgrim's</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -792,13 +770,11 @@
           <t>SVA Jean Roze</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -821,13 +797,11 @@
           <t>Savencia</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -850,13 +824,11 @@
           <t>Sicarev</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -879,13 +851,11 @@
           <t>Sodiaal</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -908,13 +878,11 @@
           <t>T'Rhea</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -937,13 +905,11 @@
           <t>Terrena</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -966,13 +932,11 @@
           <t>Van Drie</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Groupe Industriel</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1005,7 +969,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1038,7 +1001,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1071,7 +1033,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1104,7 +1065,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>Produits Laitiers</t>
@@ -1137,7 +1097,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Œufs</t>
@@ -1170,7 +1129,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1203,7 +1161,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1236,7 +1193,6 @@
           <t>Interprofession</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>Viande</t>
@@ -1259,7 +1215,6 @@
           <t>Actimel</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1292,7 +1247,6 @@
           <t>Activia</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1325,7 +1279,6 @@
           <t>Aoste</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1358,7 +1311,6 @@
           <t>Babybel</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1391,7 +1343,6 @@
           <t>Boursin</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1424,7 +1375,6 @@
           <t>Bridel</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1457,7 +1407,6 @@
           <t>Broceliande</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1490,7 +1439,6 @@
           <t>Candia</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1523,7 +1471,6 @@
           <t>Caprice des Dieux</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1556,7 +1503,6 @@
           <t>Charal</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1589,7 +1535,6 @@
           <t>Chaumes</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1622,7 +1567,6 @@
           <t>Cochonou</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1655,7 +1599,6 @@
           <t>Coeur de Lion</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1688,7 +1631,6 @@
           <t>Danette</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1721,7 +1663,6 @@
           <t>Danonino</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1754,7 +1695,6 @@
           <t>Elivia</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1787,7 +1727,6 @@
           <t>Elle &amp; Vire</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1820,7 +1759,6 @@
           <t>Entremont</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1853,7 +1791,6 @@
           <t>Fleury Michon</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1886,7 +1823,6 @@
           <t>Galbani</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1919,7 +1855,6 @@
           <t>Gastronome</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1952,7 +1887,6 @@
           <t>Gervais</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -1985,7 +1919,6 @@
           <t>Grand Fermage</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2018,7 +1951,6 @@
           <t>Herta</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2051,7 +1983,6 @@
           <t>Justin Bridou</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2084,7 +2015,6 @@
           <t>Kiri</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2117,7 +2047,6 @@
           <t>La Laitiere</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2150,7 +2079,6 @@
           <t>La Vache qui rit</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2183,7 +2111,6 @@
           <t>Lactel</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2216,7 +2143,6 @@
           <t>Le Gaulois</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2249,7 +2175,6 @@
           <t>Leerdammer</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2282,7 +2207,6 @@
           <t>Loue</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2315,7 +2239,6 @@
           <t>Maitre Coq</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2348,7 +2271,6 @@
           <t>Mamie Nova</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2381,7 +2303,6 @@
           <t>Marie</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2414,7 +2335,6 @@
           <t>Paysan Breton</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2447,7 +2367,6 @@
           <t>Pere Dodu</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2480,7 +2399,6 @@
           <t>President</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2513,7 +2431,6 @@
           <t>Regilait</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2546,7 +2463,6 @@
           <t>Sabeval</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2579,7 +2495,6 @@
           <t>Saint Agur</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2612,7 +2527,6 @@
           <t>Saint Moret</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2645,7 +2559,6 @@
           <t>Salakis</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2678,7 +2591,6 @@
           <t>Societe</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2711,7 +2623,6 @@
           <t>Socopa</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2744,7 +2655,6 @@
           <t>Soignon</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2777,7 +2687,6 @@
           <t>Taillefine</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2810,7 +2719,6 @@
           <t>Tartare</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2843,7 +2751,6 @@
           <t>Tendriade</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2876,7 +2783,6 @@
           <t>Tradival</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2909,7 +2815,6 @@
           <t>Veloute</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2942,7 +2847,6 @@
           <t>Yoplait</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>Marque</t>
@@ -2980,7 +2884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:I127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3034,6 +2938,11 @@
           <t>commentaire</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>force</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3051,7 +2960,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3070,6 +2978,11 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Chaine officielle d'ANVOL, 236 abonnes, 40 videos. Lien avec FlorianOnAir signale par Vincent.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3002,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3108,6 +3020,11 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Facebook d'ANVOL, indique sur volaille-francaise.fr.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3044,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>propose</t>
@@ -3143,7 +3059,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3161,7 +3081,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3180,6 +3099,11 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>Campagne sur volaille-francaise.fr.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3123,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3218,6 +3141,11 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Campagne sur volaille-francaise.fr.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3165,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3256,6 +3183,11 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Campagne ANVOL. Deja vue dans la moisson de la chaine YouTube (17 videos).</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3207,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3294,6 +3225,11 @@
       <c r="H8" t="inlineStr">
         <is>
           <t>Campagne sur volaille-francaise.fr.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3249,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3332,6 +3267,11 @@
       <c r="H9" t="inlineStr">
         <is>
           <t>Site institutionnel d'ANVOL.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3291,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3370,6 +3309,11 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>Site d'ANVOL.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3333,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3408,6 +3351,11 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>Site de recettes d'ANVOL.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3375,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3446,6 +3393,11 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>Site d'ANVOL.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3417,6 @@
           <t>ANVOL</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3484,6 +3435,11 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>APVF — structure de promotion citee sur volaille-francaise.fr.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3459,6 @@
           <t>Actimel</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3519,7 +3474,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3537,7 +3496,6 @@
           <t>Activia</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3553,7 +3511,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3571,7 +3533,6 @@
           <t>Aoste</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3587,7 +3548,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3605,7 +3570,6 @@
           <t>Babybel</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3621,7 +3585,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3639,7 +3607,6 @@
           <t>Boursin</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3655,7 +3622,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3673,7 +3644,6 @@
           <t>Bridel</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3689,7 +3659,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3707,7 +3681,6 @@
           <t>Broceliande</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3723,7 +3696,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3741,7 +3718,6 @@
           <t>CIFOG</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3760,6 +3736,11 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>Chaine officielle du CIFOG, 788 abonnes, 197 videos.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3760,6 @@
           <t>CIFOG</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3798,6 +3778,11 @@
       <c r="H22" t="inlineStr">
         <is>
           <t>Facebook et Twitter du CIFOG. La page Facebook a paye 81 annonces moissonnees le 27/08, dont quatre nommant @megalowfood.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3802,6 @@
           <t>CIFOG</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3836,6 +3820,11 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>Instagram, 20 900 abonnes. Trouve par Vincent le 27/08. **Doit remplacer l'alias « Le Foie Gras »**, qui designe l'aliment et a produit 91 candidats pour zero vrai (JOURNAL 38.2).</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3844,6 @@
           <t>CIFOG</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3874,6 +3862,11 @@
       <c r="H24" t="inlineStr">
         <is>
           <t>Chaine YouTube du CIFOG, indiquee sur lefoiegras.fr.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -3893,7 +3886,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -3912,6 +3904,11 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>Chaine officielle du CNIEL, 101 000 abonnes, 132 videos. UCOkKpH6tIRaNKPsNB7a3r3w</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3948,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3994,6 +3995,11 @@
           <t>Le sigle CNIEL n'apparait jamais dans les contenus.</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4011,7 +4017,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>propose</t>
@@ -4030,6 +4035,11 @@
       <c r="H28" t="inlineStr">
         <is>
           <t>RAPPORTE — StreetPress : episode sponsorise du podcast de Kameto et Zack Nani, tourne en Coree, voyage finance par le CNIEL. Alias fragile : le titre n'a aucun rapport lexical avec la filiere.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -4049,7 +4059,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4068,6 +4077,11 @@
       <c r="H29" t="inlineStr">
         <is>
           <t>Campagne COFINANCEE PAR L'UNION EUROPEENNE, contre la sedentarite. Nommee par Studio Danielle (1,74 M d'abonnes) dans deux descriptions : « en partenariat avec Les Produits Laitiers et leur campagne E</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4101,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4106,6 +4119,11 @@
       <c r="H30" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX. Amine = @Aminematue, 1,98 M d'abonnes YouTube.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4143,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4144,6 +4161,11 @@
       <c r="H31" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX. L'episode « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag » porte « En partenariat avec Les Produits Laitiers » en description — Vincent, 26/08.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4185,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4182,6 +4203,11 @@
       <c r="H32" t="inlineStr">
         <is>
           <t>Serie de videos de divertissement du CNIEL, hebergee sur produits-laitiers.com. Playlists nommant des createurs : « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag », « Mister V : les copains a</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4227,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4220,6 +4245,11 @@
       <c r="H33" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4239,7 +4269,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4258,6 +4287,11 @@
       <c r="H34" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX. Plusieurs createurs connus selon Vincent.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4311,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4296,6 +4329,11 @@
       <c r="H35" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4353,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4334,6 +4371,11 @@
       <c r="H36" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX. Loris = LORIS GIULIANO, 35 preuves fortes deja.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4395,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4372,6 +4413,11 @@
       <c r="H37" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX avec Mister V (6,53 M d'abonnes). Huit videos reperees sur la chaine YouTube du CNIEL.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4391,7 +4437,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4410,6 +4455,11 @@
       <c r="H38" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4479,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4448,6 +4497,11 @@
       <c r="H39" t="inlineStr">
         <is>
           <t>Serie LAIT'FLIX.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4521,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4483,7 +4536,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4501,7 +4558,6 @@
           <t>CNIEL</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4517,7 +4573,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4535,7 +4595,6 @@
           <t>CNPO</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4554,6 +4613,11 @@
       <c r="H42" t="inlineStr">
         <is>
           <t>Compte Instagram de la vitrine Oeufs de France, 16 700 abonnes. Trouve par Vincent le 29/08.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4637,6 @@
           <t>CNPO</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>propose</t>
@@ -4589,7 +4652,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4607,7 +4674,6 @@
           <t>Candia</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4623,7 +4689,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4641,7 +4711,6 @@
           <t>Caprice des Dieux</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4657,7 +4726,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4675,7 +4748,6 @@
           <t>Charal</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4691,7 +4763,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4709,7 +4785,6 @@
           <t>Charal (Bigard)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4728,6 +4803,11 @@
       <c r="H47" t="inlineStr">
         <is>
           <t>Second compte Charal.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4827,6 @@
           <t>Charal (Bigard)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4766,6 +4845,11 @@
       <c r="H48" t="inlineStr">
         <is>
           <t>Verifie par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4785,7 +4869,6 @@
           <t>Chaumes</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4801,7 +4884,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4819,7 +4906,6 @@
           <t>Cochonou</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4835,7 +4921,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4853,7 +4943,6 @@
           <t>Coeur de Lion</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4869,7 +4958,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4887,7 +4980,6 @@
           <t>Danette</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4903,7 +4995,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4921,7 +5017,6 @@
           <t>Danone</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>propose</t>
@@ -4940,6 +5035,11 @@
       <c r="H53" t="inlineStr">
         <is>
           <t>Seul compte Danone trouve. Vincent : « pas sur que ce soit francais ». Il n'existe PAS de @danone.france.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -4959,7 +5059,6 @@
           <t>Danonino</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -4975,7 +5074,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4993,7 +5096,6 @@
           <t>Elivia</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5009,7 +5111,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5027,7 +5133,6 @@
           <t>Elle &amp; Vire</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5043,7 +5148,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5061,7 +5170,6 @@
           <t>Entremont</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5077,7 +5185,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5095,7 +5207,6 @@
           <t>FNPSMS</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>temoin</t>
@@ -5114,6 +5225,11 @@
       <c r="H58" t="inlineStr">
         <is>
           <t>HORS PERIMETRE. Groupe temoin.</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5249,6 @@
           <t>Fleury Michon</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5149,7 +5264,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5167,7 +5286,6 @@
           <t>Galbani</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5183,7 +5301,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5201,7 +5323,6 @@
           <t>Gastronome</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5217,7 +5338,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5235,7 +5360,6 @@
           <t>Gervais</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5251,7 +5375,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5269,7 +5397,6 @@
           <t>Grand Fermage</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5285,7 +5412,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5303,7 +5434,6 @@
           <t>Herta</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5319,7 +5449,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5337,7 +5471,6 @@
           <t>Herta (Nestle)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5356,6 +5489,11 @@
       <c r="H65" t="inlineStr">
         <is>
           <t>Deja present dans les abonnements d'INAPORC, 13 contenus commerciaux TikTok.</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5513,6 @@
           <t>INAPORC</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>propose</t>
@@ -5391,7 +5528,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5409,7 +5550,6 @@
           <t>INAPORC</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5428,6 +5568,11 @@
       <c r="H67" t="inlineStr">
         <is>
           <t>RAPPORTE — Greenpeace : campagne europeenne ayant touche 74 millions de millennials en 2020.</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5592,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5466,6 +5610,11 @@
       <c r="H68" t="inlineStr">
         <is>
           <t>Chaine officielle d'INTERBEV, 79 500 abonnes, 292 videos. UCGVLdT9d5MIDrqiiMDht-jg</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5634,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5504,6 +5652,11 @@
       <c r="H69" t="inlineStr">
         <is>
           <t>Une des structures regionales. D'autres existent : Occitanie, Grand Est, Pays de la Loire — leurs comptes restent a relever.</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -5523,7 +5676,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5542,6 +5694,11 @@
       <c r="H70" t="inlineStr">
         <is>
           <t>Releve par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5718,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5580,6 +5736,11 @@
       <c r="H71" t="inlineStr">
         <is>
           <t>Releve par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5760,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5618,6 +5778,11 @@
       <c r="H72" t="inlineStr">
         <is>
           <t>Releve par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5802,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -5656,6 +5820,11 @@
       <c r="H73" t="inlineStr">
         <is>
           <t>Releve par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5864,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5733,7 +5906,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5776,6 +5953,11 @@
           <t>Seul tag de partenaire commercial apparu sur la campagne 2025, et seulement sur 1 publication sur 3.</t>
         </is>
       </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5813,7 +5995,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5851,7 +6037,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5889,7 +6079,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5927,7 +6121,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5965,7 +6163,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>fort</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6003,7 +6205,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>hashtag generique : 9 faux positifs mesures le 06/09</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6041,7 +6252,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>hashtag generique : declasse avec #Viande le 06/09</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6059,7 +6279,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6077,7 +6296,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Portes ouvertes annuelles de la filiere elevage et viande. Nommee dans les descriptions de FlorianOnAir (734 k abonnes), jugees collaborations remunerees par Vincent. Absente de la table jusqu'au 26/0</t>
+          <t>Portes ouvertes annuelles de la filiere elevage et viande. Nommee dans les descriptions de FlorianOnAir (734 k abonnes), jugees collaborations remunerees par Vincent. Absente de la table jusqu'au 26/0 | 12 faux positifs mesures le 06/09 (mentionnee sans remuneration)</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6321,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6116,6 +6339,11 @@
       <c r="H85" t="inlineStr">
         <is>
           <t>RAPPORTE — Greenpeace : serie TV, bandes dessinees et livrets, touchant 508 985 enfants de 6 a 11 ans dans 999 communes entre 2016 et 2019. Le site la-viande.fr porte une variante « Bienvenue chez les</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6363,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6154,6 +6381,11 @@
       <c r="H86" t="inlineStr">
         <is>
           <t>Presente dans une video comme un 'collectif' d'eleveurs independant. C'est le nom de la campagne Interbev, pas un collectif.</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6405,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6191,7 +6422,12 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Recuperation du mot flexitarien en 2019, vide de son sens de reduction.</t>
+          <t>Recuperation du mot flexitarien en 2019, vide de son sens de reduction. | 4 faux positifs mesures le 06/09</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6447,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6230,6 +6465,11 @@
       <c r="H88" t="inlineStr">
         <is>
           <t>RAPPORTE — Greenpeace : 7 900 salles d'attente, 22 millions de patients, 2016.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6489,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6268,6 +6507,11 @@
       <c r="H89" t="inlineStr">
         <is>
           <t>Serie sur la-viande.fr.</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6531,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6306,6 +6549,11 @@
       <c r="H90" t="inlineStr">
         <is>
           <t>Serie sur la-viande.fr. Cyril Lignac y recoit des professionnels de la filiere. Releve le 28/08.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6573,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6344,6 +6591,11 @@
       <c r="H91" t="inlineStr">
         <is>
           <t>Serie de videos sur la filiere, hebergee sur la-viande.fr. Compte @lamourboeuf deja repere dans les abonnements d'INTERBEV.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6615,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6382,6 +6633,11 @@
       <c r="H92" t="inlineStr">
         <is>
           <t>Serie sur la-viande.fr — « l'emission qui taille bavette ».</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6657,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6420,6 +6675,11 @@
       <c r="H93" t="inlineStr">
         <is>
           <t>Serie video sur la-viande.fr, relevee par Vincent.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6699,6 @@
           <t>INTERBEV</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6455,7 +6714,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6473,7 +6736,6 @@
           <t>Intercereales</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>temoin</t>
@@ -6492,6 +6754,11 @@
       <c r="H95" t="inlineStr">
         <is>
           <t>HORS PERIMETRE. Groupe temoin pour tester la detection.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6778,6 @@
           <t>Justin Bridou</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6527,7 +6793,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6545,7 +6815,6 @@
           <t>Kiri</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6561,7 +6830,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6579,7 +6852,6 @@
           <t>La Laitiere</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6595,7 +6867,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6613,7 +6889,6 @@
           <t>La Vache qui rit</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6629,7 +6904,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6647,7 +6926,6 @@
           <t>Lactel</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6663,7 +6941,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6681,7 +6963,6 @@
           <t>Le Gaulois</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6697,7 +6978,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6715,7 +7000,6 @@
           <t>Le Gaulois (LDC)</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6734,6 +7018,11 @@
       <c r="H102" t="inlineStr">
         <is>
           <t>Verifie par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6753,7 +7042,6 @@
           <t>Leerdammer</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6769,7 +7057,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6787,7 +7079,6 @@
           <t>Loue</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6803,7 +7094,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6821,7 +7116,6 @@
           <t>Maitre Coq</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6837,7 +7131,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6855,7 +7153,6 @@
           <t>Mamie Nova</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6871,7 +7168,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6889,7 +7190,6 @@
           <t>Marie</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6905,7 +7205,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6923,7 +7227,6 @@
           <t>Nature de Breton (beurre, Bretagne)</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6942,6 +7245,11 @@
       <c r="H108" t="inlineStr">
         <is>
           <t xml:space="preserve">MESURE du 29/08 : quatre videos de Lebouseuh portent la marque en description, dont « 24H A LA FERME ! » (visite de ferme et de beurrerie, 03/06/2023) et « ROADTRIP DANS LA MEILLEURE REGION DE FRANCE </t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>faible</t>
         </is>
       </c>
     </row>
@@ -6961,7 +7269,6 @@
           <t>Nestle France</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -6980,6 +7287,11 @@
       <c r="H109" t="inlineStr">
         <is>
           <t>Verifie par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -6999,7 +7311,6 @@
           <t>Paysan Breton</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7015,7 +7326,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7033,7 +7348,6 @@
           <t>Pere Dodu</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7049,7 +7363,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7067,7 +7385,6 @@
           <t>President</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7083,7 +7400,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7101,7 +7422,6 @@
           <t>Regilait</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7117,7 +7437,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7135,7 +7459,6 @@
           <t>Sabeval</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7151,7 +7474,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7169,7 +7496,6 @@
           <t>Saint Agur</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7185,7 +7511,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7203,7 +7533,6 @@
           <t>Saint Moret</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7219,7 +7548,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7237,7 +7570,6 @@
           <t>Salakis</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7253,7 +7585,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -7271,7 +7607,6 @@
           <t>Savencia</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7290,6 +7625,11 @@
       <c r="H118" t="inlineStr">
         <is>
           <t>Verifie par Vincent le 26/08.</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>fort</t>
         </is>
       </c>
     </row>
@@ -7309,7 +7649,6 @@
           <t>Societe</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7325,7 +7664,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7343,7 +7686,6 @@
           <t>Socopa</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7359,7 +7701,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7377,7 +7723,6 @@
           <t>Soignon</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7393,7 +7738,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7411,7 +7760,6 @@
           <t>Taillefine</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7427,7 +7775,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7445,7 +7797,6 @@
           <t>Tartare</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7461,7 +7812,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7479,7 +7834,6 @@
           <t>Tendriade</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7495,7 +7849,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7513,7 +7871,6 @@
           <t>Tradival</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7529,7 +7886,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7547,7 +7908,6 @@
           <t>Veloute</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7563,7 +7923,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7581,7 +7945,6 @@
           <t>Yoplait</t>
         </is>
       </c>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>confirme</t>
@@ -7597,7 +7960,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Suite aux deux notes de Vincent : indice a proximite du signal, CHAUD ! declasse
Un indice commercial ne compte plus que dans les 500 caracteres d un signal
(le << merci a >> d un autre annonceur ne valide plus des credits d equipe),
et le nom de serie CHAUD ! passe en faible. Sur le banc des 391 verdicts :
R3 a 94 % / 79 % (contre 94 / 81 sans proximite, portees 250/500/800
comparees). Reponses aux notes : recherche/recolte_jugements_2026-09-06.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -4160,12 +4160,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Serie LAIT'FLIX. L'episode « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag » porte « En partenariat avec Les Produits Laitiers » en description — Vincent, 26/08.</t>
+          <t>Serie LAIT'FLIX. L'episode « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag » porte « En partenariat avec Les Produits Laitiers » en description — Vincent, 26/08. | descendu en faible le 06/09 : accroche &lt;&lt; tres chaud ! &gt;&gt; (faux positif juge par Vincent, video AImmeZ4o13g)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>fort</t>
+          <t>faible</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Propositions integrees : 6 chaines ajoutees a la surveillance, 47 signaux en propose
Ratification en bloc par Vincent. Resolution des chaines YouTube par le
lien canonical des pages publiques (le premier channelId du HTML est celui
d une chaine recommandee — bug corrige). 39 comptes restent a resoudre,
majoritairement Instagram/TikTok : donnees/suivis_confirmes.csv

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -2884,7 +2884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I127"/>
+  <dimension ref="A1:I174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7971,6 +7971,1980 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Les Produits Laitiers</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Leporc</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>INAPORC</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Interview Métiers</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Les produits tripiers</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Label Rouge</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Histoire Métiers</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Nos Chefs nous manquent</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>MIV 2021</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>lesprolaitiers</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Made in viande 2014</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Milk Check</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Et si on en parlait</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Nos amis pour la vie</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>La Sauce de la Paix</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Génération XYZ</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>laviandetv</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Grand Voyage</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Pures sensations</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>On the road to Foie Gras</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>DANS NOS ASSIETTES</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Le lait c'est gai</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>MADE in VIANDE 2017</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Recette Cuisine Viande</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Recette de Cuisine Viande</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>XYZ Generation</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Foie Gras in pictures</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Label Rouge</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Les produits tripiers</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Fromages de France</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>CNIEL</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Viande Bio</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>I L'OVIN</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Filière viande</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Expert d'élevage</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Viande Elevage Bio</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>INTERBEV</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Foie Gras in Reels</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Foie Gras in Reels - E2</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Foie Gras in Reels - E1</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Le Foie Gras en Reels-E2</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>WEB SÉRIE CULINAIRE</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Le Magret</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Secret de Cheffe en vidéo</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Challenge Foie Gras 2014</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Foie Gras 2017</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Foie Gras</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Foie Gras et Magret</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Oies et Canards</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>CIFOG</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>LesCharcuteries</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>nom de serie ou de campagne</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>INAPORC</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>propose</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
D-marques appliquee : 52 noms de marque hors detection, bruit -97 %
3 736 -> 126 paires sur le corpus gele ; banc interprofession inchange
(94 % / 79 %). Reversible cellule par cellule dans DICTIONNAIRE.xlsx.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -3461,7 +3461,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3472,6 +3472,11 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -3498,7 +3503,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3509,6 +3514,11 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -3535,7 +3545,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3546,6 +3556,11 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -3572,7 +3587,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3583,6 +3598,11 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -3609,7 +3629,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3620,6 +3640,11 @@
       <c r="G18" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -3646,7 +3671,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3657,6 +3682,11 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -3683,7 +3713,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3694,6 +3724,11 @@
       <c r="G20" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -4676,7 +4711,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4687,6 +4722,11 @@
       <c r="G44" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4713,7 +4753,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4724,6 +4764,11 @@
       <c r="G45" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4750,7 +4795,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4761,6 +4806,11 @@
       <c r="G46" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4871,7 +4921,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -4882,6 +4932,11 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -4908,7 +4963,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4919,6 +4974,11 @@
       <c r="G50" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4945,7 +5005,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4956,6 +5016,11 @@
       <c r="G51" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4982,7 +5047,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4993,6 +5058,11 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5061,7 +5131,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -5072,6 +5142,11 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5098,7 +5173,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -5109,6 +5184,11 @@
       <c r="G55" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5135,7 +5215,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -5146,6 +5226,11 @@
       <c r="G56" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5172,7 +5257,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -5183,6 +5268,11 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5251,7 +5341,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -5262,6 +5352,11 @@
       <c r="G59" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5288,7 +5383,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5299,6 +5394,11 @@
       <c r="G60" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5325,7 +5425,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5336,6 +5436,11 @@
       <c r="G61" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5362,7 +5467,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5373,6 +5478,11 @@
       <c r="G62" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -5399,7 +5509,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5410,6 +5520,11 @@
       <c r="G63" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5436,7 +5551,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -5447,6 +5562,11 @@
       <c r="G64" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6785,7 +6905,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -6796,6 +6916,11 @@
       <c r="G96" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6822,7 +6947,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -6833,6 +6958,11 @@
       <c r="G97" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6859,7 +6989,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -6870,6 +7000,11 @@
       <c r="G98" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6896,7 +7031,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -6907,6 +7042,11 @@
       <c r="G99" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6933,7 +7073,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -6944,6 +7084,11 @@
       <c r="G100" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6970,7 +7115,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6981,6 +7126,11 @@
       <c r="G101" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -7049,7 +7199,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -7060,6 +7210,11 @@
       <c r="G103" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7086,7 +7241,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -7097,6 +7252,11 @@
       <c r="G104" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7123,7 +7283,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -7134,6 +7294,11 @@
       <c r="G105" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7160,7 +7325,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -7171,6 +7336,11 @@
       <c r="G106" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7197,7 +7367,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -7208,6 +7378,11 @@
       <c r="G107" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7318,7 +7493,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -7329,6 +7504,11 @@
       <c r="G110" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7355,7 +7535,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -7366,6 +7546,11 @@
       <c r="G111" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7392,7 +7577,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -7403,6 +7588,11 @@
       <c r="G112" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7429,7 +7619,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -7440,6 +7630,11 @@
       <c r="G113" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7466,7 +7661,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -7477,6 +7672,11 @@
       <c r="G114" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7503,7 +7703,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -7514,6 +7714,11 @@
       <c r="G115" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7540,7 +7745,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -7551,6 +7756,11 @@
       <c r="G116" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7577,7 +7787,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -7588,6 +7798,11 @@
       <c r="G117" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7656,7 +7871,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -7667,6 +7882,11 @@
       <c r="G119" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7693,7 +7913,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -7704,6 +7924,11 @@
       <c r="G120" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7730,7 +7955,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -7741,6 +7966,11 @@
       <c r="G121" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7767,7 +7997,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -7778,6 +8008,11 @@
       <c r="G122" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7804,7 +8039,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -7815,6 +8050,11 @@
       <c r="G123" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7841,7 +8081,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -7852,6 +8092,11 @@
       <c r="G124" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -7878,7 +8123,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -7889,6 +8134,11 @@
       <c r="G125" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -7915,7 +8165,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -7926,6 +8176,11 @@
       <c r="G126" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7952,7 +8207,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -7963,6 +8218,11 @@
       <c r="G127" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>retire de la detection le 06/09 (D-marques) : 0/27 mesure sur le lot de validation ; le canal marque passera par les @comptes et hashtags officiels</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">

</xml_diff>

<commit_message>
Modele de sortie, tables publiques, rescan retroactif : la boucle est complete
- MODELE_DE_SORTIE.md : le schema public defini AVANT l outil (conseil de
  la soeur de Vincent et de son ami, 06/09)
- construire_dossiers.py : 4 tables plates depuis les 84 verdicts humains
  (16 createurs, 64 CNIEL / 17 INTERBEV / 2 INAPORC / 1 ANVOL)
- rescanner_base.py : tout changement de dictionnaire est retroactif sur
  les 53 208 videos en quelques secondes
- generer_a_juger branche sur la base (corpus + tournees du facteur),
  garde-fou assoupli pour les classeurs entierement recoltes
- CHAUD ! retire de la detection (0 vrai, 3+ faux juges)
- Etat stationnaire atteint : 1 seule paire a juger, pre-triee
  collaboration probable (Nico d Estais x Nestle France via @mention)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -4180,7 +4180,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>confirme</t>
+          <t>propose</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Serie LAIT'FLIX. L'episode « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag » porte « En partenariat avec Les Produits Laitiers » en description — Vincent, 26/08. | descendu en faible le 06/09 : accroche &lt;&lt; tres chaud ! &gt;&gt; (faux positif juge par Vincent, video AImmeZ4o13g)</t>
+          <t>Serie LAIT'FLIX. L'episode « ON DEVIENT FERMIER 48H DANS LES MONTAGNES Feat Inoxtag » porte « En partenariat avec Les Produits Laitiers » en description — Vincent, 26/08. | descendu en faible le 06/09 : accroche &lt;&lt; tres chaud ! &gt;&gt; (faux positif juge par Vincent, video AImmeZ4o13g) | retire de la detection le 06/09 au soir : 0 vrai et 3+ faux positifs juges, meme en faible (recettes servez chaud)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">

</xml_diff>

<commit_message>
Evaluation des 105 signaux proposes (agent) : 6 a confirmer fort, 46 a rejeter
Chaque signal mesure sur les 53 381 videos et croise avec les verdicts.
Rapports : recherche/evaluation_signaux_proposes_2026-09-06.{csv,md}
Deux doublons du dictionnaire supprimes (Label Rouge, produits tripiers).
Les confirmations restent a Vincent (critere 11).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nAB9oA9tpiyu468RMoseS
</commit_message>
<xml_diff>
--- a/DICTIONNAIRE.xlsx
+++ b/DICTIONNAIRE.xlsx
@@ -2884,7 +2884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I174"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9326,7 +9326,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Label Rouge</t>
+          <t>Fromages de France</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -9336,7 +9336,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>INTERBEV</t>
+          <t>CNIEL</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -9368,7 +9368,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Les produits tripiers</t>
+          <t>Viande Bio</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -9410,7 +9410,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Fromages de France</t>
+          <t>I L'OVIN</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -9420,7 +9420,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CNIEL</t>
+          <t>INTERBEV</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -9452,7 +9452,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Viande Bio</t>
+          <t>Filière viande</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -9494,7 +9494,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>I L'OVIN</t>
+          <t>Expert d'élevage</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -9536,7 +9536,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Filière viande</t>
+          <t>Viande Elevage Bio</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -9578,7 +9578,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Expert d'élevage</t>
+          <t>Foie Gras in Reels</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>INTERBEV</t>
+          <t>CIFOG</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -9620,7 +9620,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Viande Elevage Bio</t>
+          <t>Foie Gras in Reels - E2</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>INTERBEV</t>
+          <t>CIFOG</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -9662,7 +9662,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Foie Gras in Reels</t>
+          <t>Foie Gras in Reels - E1</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -9704,7 +9704,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Foie Gras in Reels - E2</t>
+          <t>Le Foie Gras en Reels-E2</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -9746,7 +9746,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Foie Gras in Reels - E1</t>
+          <t>WEB SÉRIE CULINAIRE</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -9788,7 +9788,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Le Foie Gras en Reels-E2</t>
+          <t>Le Magret</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -9830,7 +9830,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>WEB SÉRIE CULINAIRE</t>
+          <t>Secret de Cheffe en vidéo</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -9872,7 +9872,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Le Magret</t>
+          <t>Challenge Foie Gras 2014</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -9914,7 +9914,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Secret de Cheffe en vidéo</t>
+          <t>Foie Gras 2017</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -9956,7 +9956,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Challenge Foie Gras 2014</t>
+          <t>Foie Gras</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -9998,7 +9998,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Foie Gras 2017</t>
+          <t>Foie Gras et Magret</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -10040,7 +10040,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Foie Gras</t>
+          <t>Oies et Canards</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -10082,7 +10082,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Foie Gras et Magret</t>
+          <t>LesCharcuteries</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -10092,7 +10092,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>CIFOG</t>
+          <t>INAPORC</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -10116,90 +10116,6 @@
         </is>
       </c>
       <c r="I172" t="inlineStr">
-        <is>
-          <t>faible</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Oies et Canards</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>nom de serie ou de campagne</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>CIFOG</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>propose</t>
-        </is>
-      </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>faible</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>LesCharcuteries</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>nom de serie ou de campagne</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>INAPORC</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>propose</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>decouverte vitrines 06/09, valide en bloc par Vincent (06/09)</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>ne detecte pas tant que non confirme signal par signal (critere 11)</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
         <is>
           <t>faible</t>
         </is>

</xml_diff>